<commit_message>
change year act template, add another func form year act, fix edit foprm
</commit_message>
<xml_diff>
--- a/back-end/mkd_works_service/api/templates/year_act/mkd_services_year_act_template.xlsx
+++ b/back-end/mkd_works_service/api/templates/year_act/mkd_services_year_act_template.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\Housing Company Services(HCS)\back-end\mkd_works_service\api\templates\year_act\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01195FF5-5DBB-4450-B892-BD9C629DAF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16978A7E-0801-48C4-A448-BA2C2A29ED4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="2" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
   <si>
     <t xml:space="preserve">приемки оказанных услуг и (или) выполненных работ по содержанию и текущему ремонту общего имущества в </t>
   </si>
@@ -148,12 +149,118 @@
   <si>
     <t>в лице  председателя Совета дома {{house_director}}, являющегося собственником квартиры № {{house_director_appartment}} с одной стороны, и {{company_name}},</t>
   </si>
+  <si>
+    <t>УТВЕРЖДЕНО приказом Министерства строительства и жилищно- коммунального хозяйства Российской Федерации от 26.10.2015 N 761/пр</t>
+  </si>
+  <si>
+    <t>Акт № {{act_num}}</t>
+  </si>
+  <si>
+    <t>приемки оказанных услуг и (или) выполненных работ по содержанию и</t>
+  </si>
+  <si>
+    <t>текущему ремонту общего имущества в многоквартирном доме</t>
+  </si>
+  <si>
+    <t>Г. Трехгорный</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        именуемые в дальнейшем "Заказчик", в лице {{ house_director }}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        являющегося собственником квартиры № {{house_director_appartment}}, находящейся в</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        данном многоквартирном доме, действующего на основании</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        Собственники помещений в многоквартирном доме, расположенном по адресу:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        456080 Челябинская область, г. Трехгорный, ул. {{street}}, д. {{street_number}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        {{ collective_direct_or_deliver_num }}, с одной стороны,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        и  {{company_name}}, именуемый  в дальнейшем "Исполнитель", в лице </t>
+  </si>
+  <si>
+    <t xml:space="preserve">        генерального директора {{company_director}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        действующего на основании  Устава, с другой стороны, совместно именуемые "Стороны", составили настоящий Акт о 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        нижеследующем:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">            1. Исполнителем предъявлены к приемке следующие оказанные на основании договора управления многоквартирным домом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       или договора оказания услуг по содержанию и (или) выполнению работ по ремонту общего имущества в многоквартирном доме</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       либо договора подряда по выполнению работ по ремонту общего имущества в многоквартирном доме (указать нужное)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> {{act_date}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       выполненные работы по содержанию и текущему ремонту общего имущества в многоквартирном доме № {{street_number}},</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       №   _   от "       "       г. (далее - "Договор") услуги и (или)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       расположенном по адресу: г. Трехгорный, ул. {{ street }}</t>
+  </si>
+  <si>
+    <t>Периодичность/количественн ый показатель выполненной работы (оказанной услуги)</t>
+  </si>
+  <si>
+    <t>Единица измерения работы (услуги)</t>
+  </si>
+  <si>
+    <t>Стоимость/сметна я стоимость выполненной работы (оказанной услуги) за месяц</t>
+  </si>
+  <si>
+    <t>Цена выполненной работы (оказанной услуги), в рублях</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        {{ all_work_sum }} руб.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         4. Претензий по выполнению условий Договора Стороны друг к другу не имеют. Настоящий Акт составлен в</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       2 экземплярах, имеющих одинаковую юридическую силу, по одному для каждой из Сторон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         3. Работы (услуги) выполнены (оказаны) полностью, в установленные сроки, с надлежащим качеством. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">         2. Всего за период с {{ start_work_date }} по {{ end_work_date }} выполнено работ (оказано услуг) на общую сумму</t>
+  </si>
+  <si>
+    <t>Подписи Сторон:</t>
+  </si>
+  <si>
+    <t>(подпись)</t>
+  </si>
+  <si>
+    <t>Исполнитель -              Генеральный директор  {{company_director}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заказчик -                     </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +307,13 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -236,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -249,10 +363,39 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -607,104 +750,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
@@ -760,18 +903,414 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A10:F10"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="67" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CC7D1CE-6879-4716-A847-0AFCA559B6AB}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="58.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37" s="5"/>
+    </row>
+    <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D40" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="68" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>